<commit_message>
1000 ship tests updated, need to add logging
</commit_message>
<xml_diff>
--- a/researchQuestions/test1_1_simulation_results.xlsx
+++ b/researchQuestions/test1_1_simulation_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Simulation Parameters</t>
   </si>
@@ -52,13 +52,49 @@
     <t>Truth Working, Sensed Working</t>
   </si>
   <si>
+    <t>(1, 'bad')</t>
+  </si>
+  <si>
+    <t>(1, 'moderate')</t>
+  </si>
+  <si>
+    <t>(1, 'good')</t>
+  </si>
+  <si>
+    <t>(3, 'bad')</t>
+  </si>
+  <si>
+    <t>(3, 'moderate')</t>
+  </si>
+  <si>
     <t>(3, 'good')</t>
   </si>
   <si>
-    <t>(4, 'good')</t>
+    <t>(5, 'bad')</t>
+  </si>
+  <si>
+    <t>(5, 'moderate')</t>
   </si>
   <si>
     <t>(5, 'good')</t>
+  </si>
+  <si>
+    <t>(7, 'bad')</t>
+  </si>
+  <si>
+    <t>(7, 'moderate')</t>
+  </si>
+  <si>
+    <t>(7, 'good')</t>
+  </si>
+  <si>
+    <t>(11, 'bad')</t>
+  </si>
+  <si>
+    <t>(11, 'moderate')</t>
+  </si>
+  <si>
+    <t>(11, 'good')</t>
   </si>
 </sst>
 </file>
@@ -416,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -462,37 +498,37 @@
         <v>12</v>
       </c>
       <c r="B2">
-        <v>331</v>
+        <v>0.0423495145631068</v>
       </c>
       <c r="C2">
-        <v>390</v>
+        <v>0.9576504854368934</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>0.04095977808599168</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>9.70873786407767E-06</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>9.333333333333334</v>
+        <v>0.008547850208044383</v>
       </c>
       <c r="H2">
-        <v>4.666666666666667</v>
+        <v>2.773925104022192E-06</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
-        <v>380.6666666666667</v>
+        <v>0.9488002773925105</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>0.0002926490984743412</v>
       </c>
       <c r="L2">
-        <v>326.3333333333333</v>
+        <v>0.001386962552011096</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -500,37 +536,37 @@
         <v>13</v>
       </c>
       <c r="B3">
-        <v>331</v>
+        <v>0.04277392510402219</v>
       </c>
       <c r="C3">
-        <v>390</v>
+        <v>0.9572260748959778</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>0.04086130374479889</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>0.0001081830790568655</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>9.333333333333334</v>
+        <v>0.008309292649098474</v>
       </c>
       <c r="H3">
-        <v>4.666666666666667</v>
+        <v>0.0002413314840499306</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3">
-        <v>380.6666666666667</v>
+        <v>0.9215214979195562</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>0.0272871012482663</v>
       </c>
       <c r="L3">
-        <v>326.3333333333333</v>
+        <v>0.00167128987517337</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -538,13 +574,13 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>721</v>
+        <v>0.9887766990291262</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>0.01122330097087379</v>
       </c>
       <c r="D4">
-        <v>195</v>
+        <v>0.04096948682385576</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -553,22 +589,478 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>6.38002773925104E-05</v>
       </c>
       <c r="H4">
-        <v>9.333333333333334</v>
+        <v>0.008486823855755894</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>0.005631067961165048</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>0.005528432732316227</v>
       </c>
       <c r="L4">
-        <v>516.6666666666666</v>
+        <v>0.9393203883495146</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>0.04232316227461858</v>
+      </c>
+      <c r="C5">
+        <v>0.9576768377253814</v>
+      </c>
+      <c r="D5">
+        <v>0.04082246879334257</v>
+      </c>
+      <c r="E5">
+        <v>0.0001470180305131761</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0.008457697642163661</v>
+      </c>
+      <c r="H5">
+        <v>9.292649098474341E-05</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0.9394840499306518</v>
+      </c>
+      <c r="K5">
+        <v>0.009588072122052703</v>
+      </c>
+      <c r="L5">
+        <v>0.001407766990291262</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>0.1382926490984743</v>
+      </c>
+      <c r="C6">
+        <v>0.8617073509015256</v>
+      </c>
+      <c r="D6">
+        <v>0.04035783633841886</v>
+      </c>
+      <c r="E6">
+        <v>0.0004840499306518724</v>
+      </c>
+      <c r="F6">
+        <v>0.0001276005547850208</v>
+      </c>
+      <c r="G6">
+        <v>0.005675450762829403</v>
+      </c>
+      <c r="H6">
+        <v>0.00283495145631068</v>
+      </c>
+      <c r="I6">
+        <v>4.022191400832178E-05</v>
+      </c>
+      <c r="J6">
+        <v>0.6238862690707351</v>
+      </c>
+      <c r="K6">
+        <v>0.231493758668516</v>
+      </c>
+      <c r="L6">
+        <v>0.09509986130374479</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7">
+        <v>0.9889708737864078</v>
+      </c>
+      <c r="C7">
+        <v>0.01102912621359223</v>
+      </c>
+      <c r="D7">
+        <v>0.04096948682385576</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>6.38002773925104E-05</v>
+      </c>
+      <c r="H7">
+        <v>0.008486823855755894</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0.005535367545076283</v>
+      </c>
+      <c r="K7">
+        <v>0.00542995839112344</v>
+      </c>
+      <c r="L7">
+        <v>0.9395145631067962</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8">
+        <v>0.04229126213592233</v>
+      </c>
+      <c r="C8">
+        <v>0.9577087378640776</v>
+      </c>
+      <c r="D8">
+        <v>0.04020665742024965</v>
+      </c>
+      <c r="E8">
+        <v>0.0007628294036061027</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0.008011095700416089</v>
+      </c>
+      <c r="H8">
+        <v>0.0005395284327323163</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0.8935991678224687</v>
+      </c>
+      <c r="K8">
+        <v>0.05533564493758669</v>
+      </c>
+      <c r="L8">
+        <v>0.001545076282940361</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9">
+        <v>0.4226546463245492</v>
+      </c>
+      <c r="C9">
+        <v>0.5773453536754507</v>
+      </c>
+      <c r="D9">
+        <v>0.04036754507628294</v>
+      </c>
+      <c r="E9">
+        <v>0.0004479889042995839</v>
+      </c>
+      <c r="F9">
+        <v>0.0001539528432732316</v>
+      </c>
+      <c r="G9">
+        <v>0.002699029126213592</v>
+      </c>
+      <c r="H9">
+        <v>0.005776699029126213</v>
+      </c>
+      <c r="I9">
+        <v>7.489597780859917E-05</v>
+      </c>
+      <c r="J9">
+        <v>0.2973633841886269</v>
+      </c>
+      <c r="K9">
+        <v>0.2766061026352288</v>
+      </c>
+      <c r="L9">
+        <v>0.3765104022191401</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10">
+        <v>0.9889708737864078</v>
+      </c>
+      <c r="C10">
+        <v>0.01102912621359223</v>
+      </c>
+      <c r="D10">
+        <v>0.04096948682385576</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>6.38002773925104E-05</v>
+      </c>
+      <c r="H10">
+        <v>0.008486823855755894</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0.005535367545076283</v>
+      </c>
+      <c r="K10">
+        <v>0.00542995839112344</v>
+      </c>
+      <c r="L10">
+        <v>0.9395145631067962</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11">
+        <v>0.04255062413314841</v>
+      </c>
+      <c r="C11">
+        <v>0.9574493758668516</v>
+      </c>
+      <c r="D11">
+        <v>0.04069070735090153</v>
+      </c>
+      <c r="E11">
+        <v>0.0002773925104022191</v>
+      </c>
+      <c r="F11">
+        <v>1.386962552011096E-06</v>
+      </c>
+      <c r="G11">
+        <v>0.008262135922330096</v>
+      </c>
+      <c r="H11">
+        <v>0.0002884882108183079</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0.9184341192787795</v>
+      </c>
+      <c r="K11">
+        <v>0.0304743411927878</v>
+      </c>
+      <c r="L11">
+        <v>0.001571428571428571</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12">
+        <v>0.6362718446601943</v>
+      </c>
+      <c r="C12">
+        <v>0.3637281553398058</v>
+      </c>
+      <c r="D12">
+        <v>0.0407004160887656</v>
+      </c>
+      <c r="E12">
+        <v>0.000188626907073509</v>
+      </c>
+      <c r="F12">
+        <v>8.044382801664356E-05</v>
+      </c>
+      <c r="G12">
+        <v>0.001787794729542302</v>
+      </c>
+      <c r="H12">
+        <v>0.006728155339805825</v>
+      </c>
+      <c r="I12">
+        <v>3.467406380027739E-05</v>
+      </c>
+      <c r="J12">
+        <v>0.1937170596393897</v>
+      </c>
+      <c r="K12">
+        <v>0.1679195561719833</v>
+      </c>
+      <c r="L12">
+        <v>0.5888432732316228</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13">
+        <v>0.9889708737864078</v>
+      </c>
+      <c r="C13">
+        <v>0.01102912621359223</v>
+      </c>
+      <c r="D13">
+        <v>0.04096948682385576</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>6.38002773925104E-05</v>
+      </c>
+      <c r="H13">
+        <v>0.008486823855755894</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0.005535367545076283</v>
+      </c>
+      <c r="K13">
+        <v>0.00542995839112344</v>
+      </c>
+      <c r="L13">
+        <v>0.9395145631067962</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14">
+        <v>0.04513592233009708</v>
+      </c>
+      <c r="C14">
+        <v>0.9548640776699029</v>
+      </c>
+      <c r="D14">
+        <v>0.04035922330097087</v>
+      </c>
+      <c r="E14">
+        <v>0.0006019417475728155</v>
+      </c>
+      <c r="F14">
+        <v>8.321775312066574E-06</v>
+      </c>
+      <c r="G14">
+        <v>0.007686546463245492</v>
+      </c>
+      <c r="H14">
+        <v>0.0008626907073509015</v>
+      </c>
+      <c r="I14">
+        <v>1.386962552011096E-06</v>
+      </c>
+      <c r="J14">
+        <v>0.8512621359223301</v>
+      </c>
+      <c r="K14">
+        <v>0.09530374479889042</v>
+      </c>
+      <c r="L14">
+        <v>0.003914008321775312</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15">
+        <v>0.890755894590846</v>
+      </c>
+      <c r="C15">
+        <v>0.109244105409154</v>
+      </c>
+      <c r="D15">
+        <v>0.04088488210818308</v>
+      </c>
+      <c r="E15">
+        <v>5.131761442441054E-05</v>
+      </c>
+      <c r="F15">
+        <v>3.32871012482663E-05</v>
+      </c>
+      <c r="G15">
+        <v>0.0005131761442441054</v>
+      </c>
+      <c r="H15">
+        <v>0.008023578363384189</v>
+      </c>
+      <c r="I15">
+        <v>1.386962552011096E-05</v>
+      </c>
+      <c r="J15">
+        <v>0.05261026352288489</v>
+      </c>
+      <c r="K15">
+        <v>0.05602219140083218</v>
+      </c>
+      <c r="L15">
+        <v>0.8418474341192788</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16">
+        <v>0.9889708737864078</v>
+      </c>
+      <c r="C16">
+        <v>0.01102912621359223</v>
+      </c>
+      <c r="D16">
+        <v>0.04096948682385576</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>6.38002773925104E-05</v>
+      </c>
+      <c r="H16">
+        <v>0.008486823855755894</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0.005535367545076283</v>
+      </c>
+      <c r="K16">
+        <v>0.00542995839112344</v>
+      </c>
+      <c r="L16">
+        <v>0.9395145631067962</v>
       </c>
     </row>
   </sheetData>

</xml_diff>